<commit_message>
add new CNN LSTM model
</commit_message>
<xml_diff>
--- a/Datasets/Real Breakdown Records - Overlock.xlsx
+++ b/Datasets/Real Breakdown Records - Overlock.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Courses\IIT\AIDS\FYP\Real Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C60D031-5004-4F5C-9DD3-0E912F55D420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E4C7A66-3C54-4F36-B8E2-ABD098920526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{FE3539FE-E0B8-4DFA-B6A7-015537647EDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Id</t>
   </si>
@@ -89,6 +89,9 @@
     <t>epochT</t>
   </si>
   <si>
+    <t>Breakdown</t>
+  </si>
+  <si>
     <t>Solution Given</t>
   </si>
   <si>
@@ -131,14 +134,17 @@
     <t>Sharpen the blade</t>
   </si>
   <si>
-    <t>Breakdown</t>
+    <t>10,457,20,410,30,1313,40,1493,50,147,60,227,70,319,80,388,90,303,100,299,110,539,120,328,130,471,140,383,150,348,160,449,170,419,180,516,190,717,200,527,210,314,220,186,230,416,240,234,250,231,260,249,270,216,280,192,290,305,300,298,310,388,320,331,330,633,340,547,350,493,360,387,370,181,380,154,390,356,400,363,410,295,420,173,430,133,440,169,450,270,460,231,470,350,480,115,490,306,500,243,510,270,520,336,530,525,540,582,550,754,560,216,570,179,580,141,590,261,600,246</t>
+  </si>
+  <si>
+    <t>10,315,20,2172,30,346,40,549,50,292,60,224,70,306,80,236,90,215,100,245,110,232,120,229,130,222,140,279,150,230,160,287,170,363,180,543,190,485,200,371,210,290,220,262,230,331,240,287,250,215,260,195,270,169,280,185,290,201,300,131,310,178,320,248,330,227,340,230,350,320,360,495,370,472,380,370,390,496,400,355,410,386,420,366,430,424,440,525,450,519,460,427,470,340,480,247,490,576,500,255,510,404,520,393,530,272,540,197,550,230,560,220,570,157,580,153,590,251,600,171</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,7 +181,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -208,39 +214,212 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
-      <right style="thin">
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color theme="4" tint="0.39997558519241921"/>
-      </right>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="47" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="29" formatCode="mm:ss.0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -251,6 +430,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A6C86173-FC1B-42BB-BCDD-646423E4631B}" name="Table1" displayName="Table1" ref="A1:S8" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21" headerRowBorderDxfId="19" tableBorderDxfId="20">
+  <autoFilter ref="A1:S8" xr:uid="{A6C86173-FC1B-42BB-BCDD-646423E4631B}"/>
+  <tableColumns count="19">
+    <tableColumn id="1" xr3:uid="{084BEDB1-23FD-4763-9FDC-734B1435C2A0}" name="Id" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{DE8208D1-8884-4F55-9E56-011ABFFF885C}" name="machineRPM" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{D37592D8-99CB-4898-AE27-744D857C73BF}" name="machineVibration" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{B464EE88-ABA2-4C6A-8A88-32534006669B}" name="needleRuntime" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{68B9EEF3-B451-471F-A95A-916155D9EB30}" name="dateTime" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{8D15A975-C4D6-41A7-A43A-E489BCA55376}" name="machineSerialNumber" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{4AD7EB23-A5CC-45BA-933F-315532DBAADD}" name="status" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{B3646777-E35B-4334-B240-1A921A1AAD0B}" name="machineVoltageMean" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{1E9B2F95-0B78-4250-808C-F6014CDE45B3}" name="machineVoltageMin" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{0BBA8320-1296-4F5D-8477-F1983B4964AD}" name="machineVoltageMax" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{CC6947D0-56D7-4046-B0A2-044F4325160B}" name="machineCurrentMean" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{6571473C-2BBE-4CE2-B13A-63A9D97C588C}" name="machineCurrentMin" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{5DCF242E-E9A8-4286-BD76-FEEB9AE30343}" name="machineCurrentMax" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{C59B7660-FF72-4591-93DD-1FF3B136BD6B}" name="machinePowerMean" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{61B9ACCC-87B0-4AFC-A2B9-6743113AE98F}" name="machinePowerMin" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{23BDDCEE-A876-44CB-9632-B7DAF9A18F12}" name="machinePowerMax" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{8AA805C2-D933-45CE-84C8-8B9618EEC975}" name="epochT" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{CCC19E6C-BA33-439C-9B27-E9C5F37A2755}" name="Breakdown" dataDxfId="1"/>
+    <tableColumn id="19" xr3:uid="{F223E369-6191-466F-BB76-1D47C944CEC9}" name="Solution Given" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -570,310 +777,513 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0932AA2-3A9F-4BEA-8CF2-E9BF74B07D8F}">
-  <dimension ref="A1:S5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.140625" customWidth="1"/>
+    <col min="12" max="12" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="37.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="A2" s="1">
+        <v>276538</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5675</v>
+      </c>
+      <c r="E2" s="8">
+        <v>46072.419398148151</v>
+      </c>
+      <c r="F2" s="2">
+        <v>521760</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="2">
+        <v>230.1385956</v>
+      </c>
+      <c r="I2" s="2">
+        <v>229.51675420000001</v>
+      </c>
+      <c r="J2" s="2">
+        <v>231.71218870000001</v>
+      </c>
+      <c r="K2" s="2">
+        <v>2.3269917960000002</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.171203673</v>
+      </c>
+      <c r="M2" s="2">
+        <v>3.57053113</v>
+      </c>
+      <c r="N2" s="2">
+        <v>535.53062390416096</v>
+      </c>
+      <c r="O2" s="2">
+        <v>39.294111334078103</v>
+      </c>
+      <c r="P2" s="2">
+        <v>827.33558295378396</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>1771495435</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="1">
+        <v>276546</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="2">
+        <v>4414</v>
+      </c>
+      <c r="E3" s="8">
+        <v>46072.424108796295</v>
+      </c>
+      <c r="F3" s="2">
+        <v>521760</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2">
+        <v>228.550354</v>
+      </c>
+      <c r="I3" s="2">
+        <v>228.0391846</v>
+      </c>
+      <c r="J3" s="2">
+        <v>229.5373993</v>
+      </c>
+      <c r="K3" s="2">
+        <v>2.038337946</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.28483066000000001</v>
+      </c>
+      <c r="M3" s="2">
+        <v>2.580099583</v>
+      </c>
+      <c r="N3" s="2">
+        <v>465.86285912993202</v>
+      </c>
+      <c r="O3" s="2">
+        <v>64.952551455479806</v>
+      </c>
+      <c r="P3" s="2">
+        <v>592.22934821683396</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>1771495842</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="43.5">
+      <c r="A4" s="1">
+        <v>276547</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5597</v>
+      </c>
+      <c r="E4" s="8">
+        <v>46072.428113425929</v>
+      </c>
+      <c r="F4" s="2">
+        <v>521760</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2">
+        <v>229.50285339999999</v>
+      </c>
+      <c r="I4" s="2">
+        <v>228.70074460000001</v>
+      </c>
+      <c r="J4" s="2">
+        <v>230.4544373</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1.788824081</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.36456116999999999</v>
+      </c>
+      <c r="M4" s="2">
+        <v>3.2619428629999998</v>
+      </c>
+      <c r="N4" s="2">
+        <v>410.54023082013202</v>
+      </c>
+      <c r="O4" s="2">
+        <v>83.375411031247097</v>
+      </c>
+      <c r="P4" s="2">
+        <v>751.72920699741496</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>1771496188</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="1">
+        <v>277850</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="2">
+        <v>3626</v>
+      </c>
+      <c r="E5" s="8">
+        <v>46073.469375000001</v>
+      </c>
+      <c r="F5" s="2">
+        <v>521760</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2">
+        <v>228.34948729999999</v>
+      </c>
+      <c r="I5" s="2">
+        <v>227.24067690000001</v>
+      </c>
+      <c r="J5" s="2">
+        <v>229.21278380000001</v>
+      </c>
+      <c r="K5" s="2">
+        <v>2.2927103039999999</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.25478029299999999</v>
+      </c>
+      <c r="M5" s="2">
+        <v>4.0547394749999999</v>
+      </c>
+      <c r="N5" s="2">
+        <v>523.53922244582702</v>
+      </c>
+      <c r="O5" s="2">
+        <v>57.896446242100303</v>
+      </c>
+      <c r="P5" s="2">
+        <v>929.39812264850002</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>1771586153</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="3" t="s">
-        <v>17</v>
-      </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>276538</v>
-      </c>
-      <c r="B2" s="5">
+    <row r="6" spans="1:19">
+      <c r="A6" s="4">
+        <v>276547</v>
+      </c>
+      <c r="B6" s="4">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="5">
-        <v>5675</v>
-      </c>
-      <c r="E2" s="6">
-        <v>46072.41939920139</v>
-      </c>
-      <c r="F2" s="5">
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="4">
+        <v>5597</v>
+      </c>
+      <c r="E6" s="9">
+        <v>46072.428113425929</v>
+      </c>
+      <c r="F6" s="4">
         <v>521760</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="5">
-        <v>230.1385956</v>
-      </c>
-      <c r="I2" s="5">
-        <v>229.51675420000001</v>
-      </c>
-      <c r="J2" s="5">
-        <v>231.71218870000001</v>
-      </c>
-      <c r="K2" s="5">
-        <v>2.3269917960000002</v>
-      </c>
-      <c r="L2" s="5">
-        <v>0.171203673</v>
-      </c>
-      <c r="M2" s="5">
-        <v>3.57053113</v>
-      </c>
-      <c r="N2" s="5">
-        <v>535.53062390416096</v>
-      </c>
-      <c r="O2" s="5">
-        <v>39.294111334078103</v>
-      </c>
-      <c r="P2" s="5">
-        <v>827.33558295378396</v>
-      </c>
-      <c r="Q2" s="5">
-        <v>1771495435</v>
-      </c>
-      <c r="R2" s="5" t="s">
+      <c r="G6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="7" t="s">
-        <v>21</v>
+      <c r="H6" s="4">
+        <v>229.50285339999999</v>
+      </c>
+      <c r="I6" s="4">
+        <v>228.70074460000001</v>
+      </c>
+      <c r="J6" s="4">
+        <v>230.4544373</v>
+      </c>
+      <c r="K6" s="4">
+        <v>1.788824081</v>
+      </c>
+      <c r="L6" s="4">
+        <v>0.36456116999999999</v>
+      </c>
+      <c r="M6" s="4">
+        <v>3.2619428629999998</v>
+      </c>
+      <c r="N6" s="4">
+        <v>410.54023082013202</v>
+      </c>
+      <c r="O6" s="4">
+        <v>83.375411031247097</v>
+      </c>
+      <c r="P6" s="4">
+        <v>751.72920699741496</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>1771496188</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>276546</v>
-      </c>
-      <c r="B3" s="5">
+    <row r="7" spans="1:19">
+      <c r="A7" s="4">
+        <v>276550</v>
+      </c>
+      <c r="B7" s="4">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="5">
-        <v>4414</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46072.424113946756</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1277</v>
+      </c>
+      <c r="E7" s="9">
+        <v>46072.457604166666</v>
+      </c>
+      <c r="F7" s="4">
         <v>521760</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="5">
-        <v>228.550354</v>
-      </c>
-      <c r="I3" s="5">
-        <v>228.0391846</v>
-      </c>
-      <c r="J3" s="5">
-        <v>229.5373993</v>
-      </c>
-      <c r="K3" s="5">
-        <v>2.038337946</v>
-      </c>
-      <c r="L3" s="5">
-        <v>0.28483066000000001</v>
-      </c>
-      <c r="M3" s="5">
-        <v>2.580099583</v>
-      </c>
-      <c r="N3" s="5">
-        <v>465.86285912993202</v>
-      </c>
-      <c r="O3" s="5">
-        <v>64.952551455479806</v>
-      </c>
-      <c r="P3" s="5">
-        <v>592.22934821683396</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>1771495842</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="S3" s="7" t="s">
+      <c r="G7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="4">
+        <v>231.44932560000001</v>
+      </c>
+      <c r="I7" s="4">
+        <v>231.03732299999999</v>
+      </c>
+      <c r="J7" s="4">
+        <v>231.72172549999999</v>
+      </c>
+      <c r="K7" s="4">
+        <v>0.80958849200000005</v>
+      </c>
+      <c r="L7" s="4">
+        <v>0.16418586700000001</v>
+      </c>
+      <c r="M7" s="4">
+        <v>1.5467116830000001</v>
+      </c>
+      <c r="N7" s="4">
+        <v>187.37871048692099</v>
+      </c>
+      <c r="O7" s="4">
+        <v>37.933063186113998</v>
+      </c>
+      <c r="P7" s="4">
+        <v>358.40670003576901</v>
+      </c>
+      <c r="Q7" s="4">
+        <v>1771498736</v>
+      </c>
+      <c r="R7" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="S7" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="4" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>276547</v>
-      </c>
-      <c r="B4" s="5">
+    <row r="8" spans="1:19">
+      <c r="A8" s="4">
+        <v>276549</v>
+      </c>
+      <c r="B8" s="4">
         <v>0</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="4">
+        <v>4052</v>
+      </c>
+      <c r="E8" s="9">
+        <v>46072.45752314815</v>
+      </c>
+      <c r="F8" s="4">
+        <v>521760</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="4">
+        <v>231.8682556</v>
+      </c>
+      <c r="I8" s="4">
+        <v>231.3586731</v>
+      </c>
+      <c r="J8" s="4">
+        <v>232.33648679999999</v>
+      </c>
+      <c r="K8" s="4">
+        <v>0.84228324899999996</v>
+      </c>
+      <c r="L8" s="4">
+        <v>0.25146970200000002</v>
+      </c>
+      <c r="M8" s="4">
+        <v>0.90254420000000002</v>
+      </c>
+      <c r="N8" s="4">
+        <v>195.29874766673001</v>
+      </c>
+      <c r="O8" s="4">
+        <v>58.179696579572401</v>
+      </c>
+      <c r="P8" s="4">
+        <v>209.69394860971599</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>1771498729</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="S8" s="7" t="s">
         <v>25</v>
-      </c>
-      <c r="D4" s="5">
-        <v>5597</v>
-      </c>
-      <c r="E4" s="6">
-        <v>46072.428112106485</v>
-      </c>
-      <c r="F4" s="5">
-        <v>521760</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="5">
-        <v>229.50285339999999</v>
-      </c>
-      <c r="I4" s="5">
-        <v>228.70074460000001</v>
-      </c>
-      <c r="J4" s="5">
-        <v>230.4544373</v>
-      </c>
-      <c r="K4" s="5">
-        <v>1.788824081</v>
-      </c>
-      <c r="L4" s="5">
-        <v>0.36456116999999999</v>
-      </c>
-      <c r="M4" s="5">
-        <v>3.2619428629999998</v>
-      </c>
-      <c r="N4" s="5">
-        <v>410.54023082013202</v>
-      </c>
-      <c r="O4" s="5">
-        <v>83.375411031247097</v>
-      </c>
-      <c r="P4" s="5">
-        <v>751.72920699741496</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>1771496188</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="S4" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>277850</v>
-      </c>
-      <c r="B5" s="5">
-        <v>0</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="5">
-        <v>3626</v>
-      </c>
-      <c r="E5" s="6">
-        <v>46073.469376805559</v>
-      </c>
-      <c r="F5" s="5">
-        <v>521760</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="5">
-        <v>228.34948729999999</v>
-      </c>
-      <c r="I5" s="5">
-        <v>227.24067690000001</v>
-      </c>
-      <c r="J5" s="5">
-        <v>229.21278380000001</v>
-      </c>
-      <c r="K5" s="5">
-        <v>2.2927103039999999</v>
-      </c>
-      <c r="L5" s="5">
-        <v>0.25478029299999999</v>
-      </c>
-      <c r="M5" s="5">
-        <v>4.0547394749999999</v>
-      </c>
-      <c r="N5" s="5">
-        <v>523.53922244582702</v>
-      </c>
-      <c r="O5" s="5">
-        <v>57.896446242100303</v>
-      </c>
-      <c r="P5" s="5">
-        <v>929.39812264850002</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>1771586153</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 MAS | MAS Only</oddFooter>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{af926f27-653d-49b5-a458-2176741aa4ba}" enabled="1" method="Standard" siteId="{852c5799-8134-4f15-9d38-eba4296cc76f}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>